<commit_message>
feat(relatorios): criar dashboards formatados no excel e atualizar regras de tarifas e suporte operacional
</commit_message>
<xml_diff>
--- a/gestao_projetos/execucao_financeira/execucao_financeira.xlsx
+++ b/gestao_projetos/execucao_financeira/execucao_financeira.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ARGUS\gestao_projetos\execucao_financeira\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A55C569-FA39-4D96-8A6F-52A7E5359313}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71D87D72-B451-4084-9CB3-0DF0561CB703}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{49823ED3-3B2F-469D-97DF-36A3ABB00E6B}"/>
   </bookViews>
@@ -21,7 +21,7 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="1" r:id="rId3"/>
+    <pivotCache cacheId="0" r:id="rId3"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -1644,7 +1644,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{9DB36DD7-534E-4BAC-8DEA-04C59BA20F0E}" name="Tabela dinâmica4" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{9DB36DD7-534E-4BAC-8DEA-04C59BA20F0E}" name="Tabela dinâmica4" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Valores" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A3:B27" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="9">
     <pivotField axis="axisRow" showAll="0" sortType="ascending" defaultSubtotal="0">
@@ -2176,7 +2176,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" ht="45" hidden="1" x14ac:dyDescent="0.25">
       <c r="A2" s="5">
         <v>46204</v>
       </c>
@@ -2209,7 +2209,7 @@
         <v>27500</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="60" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3" s="5">
         <v>46210</v>
       </c>
@@ -2242,7 +2242,7 @@
         <v>-1375</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" ht="75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A4" s="5">
         <v>46213</v>
       </c>
@@ -2506,7 +2506,7 @@
         <v>-12.34</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="5">
         <v>46219</v>
       </c>
@@ -2539,7 +2539,7 @@
         <v>-2800</v>
       </c>
     </row>
-    <row r="13" spans="1:10" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A13" s="5">
         <v>46239</v>
       </c>
@@ -2572,7 +2572,7 @@
         <v>-2800</v>
       </c>
     </row>
-    <row r="14" spans="1:10" ht="30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:10" ht="30" x14ac:dyDescent="0.25">
       <c r="A14" s="5">
         <v>46273</v>
       </c>
@@ -2605,7 +2605,7 @@
         <v>-2800</v>
       </c>
     </row>
-    <row r="15" spans="1:10" ht="60" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:10" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A15" s="5">
         <v>46254</v>
       </c>
@@ -2638,7 +2638,7 @@
         <v>-128.58000000000001</v>
       </c>
     </row>
-    <row r="16" spans="1:10" ht="60" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A16" s="5">
         <v>46281</v>
       </c>
@@ -3067,7 +3067,7 @@
         <v>-200.93</v>
       </c>
     </row>
-    <row r="29" spans="1:10" ht="60" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:10" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A29" s="5">
         <v>46210</v>
       </c>
@@ -4486,7 +4486,7 @@
         <v>-32.07</v>
       </c>
     </row>
-    <row r="72" spans="1:10" ht="60" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:10" ht="60" hidden="1" x14ac:dyDescent="0.25">
       <c r="A72" s="5">
         <v>46189</v>
       </c>
@@ -4929,10 +4929,11 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:J84" xr:uid="{E3F049E5-0281-4D5D-A75B-91688D40DD5E}">
-    <filterColumn colId="7">
+    <filterColumn colId="8">
       <filters>
-        <filter val="Entrada de Receita"/>
-        <filter val="Transferência entre Projetos"/>
+        <filter val="Pagamento bolsa para Geziel Sena Colares, 83403876268, referente à parcela 01/08."/>
+        <filter val="Pagamento bolsa para Geziel Sena Colares, 83403876268, referente à parcela 02/08."/>
+        <filter val="Pagamento bolsa para Geziel Sena Colares, 83403876268, referente à parcela 03/08."/>
       </filters>
     </filterColumn>
   </autoFilter>

</xml_diff>